<commit_message>
test 4 banner store / map.ed
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/neutralC.xlsx
+++ b/gu_in/Map.edf/neutralC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B026C84C-356E-4C87-9A83-C2B984F3DABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A54DC82D-7723-4D29-BA15-1FA79B8D3DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10965" yWindow="1020" windowWidth="10110" windowHeight="11205" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3092" uniqueCount="1489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3100" uniqueCount="1497">
   <si>
     <t>char[32]</t>
   </si>
@@ -4505,6 +4505,30 @@
   </si>
   <si>
     <t>bd131B2</t>
+  </si>
+  <si>
+    <t>sd131B7</t>
+  </si>
+  <si>
+    <t>bd131B7</t>
+  </si>
+  <si>
+    <t>sd131B8</t>
+  </si>
+  <si>
+    <t>bd131B8</t>
+  </si>
+  <si>
+    <t>sd131B9</t>
+  </si>
+  <si>
+    <t>bd131B9</t>
+  </si>
+  <si>
+    <t>sd131C0</t>
+  </si>
+  <si>
+    <t>bd131C0</t>
   </si>
 </sst>
 </file>
@@ -46681,7 +46705,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H215"/>
+  <dimension ref="A1:H223"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="9.7109375" customWidth="1"/>
@@ -52274,6 +52298,214 @@
         <v>20</v>
       </c>
       <c r="H215" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8">
+      <c r="A216" s="1" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B216" s="1">
+        <v>106</v>
+      </c>
+      <c r="C216" s="1">
+        <v>7489</v>
+      </c>
+      <c r="D216" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E216" s="1">
+        <v>508</v>
+      </c>
+      <c r="F216" s="1">
+        <v>20</v>
+      </c>
+      <c r="G216" s="1">
+        <v>20</v>
+      </c>
+      <c r="H216" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8">
+      <c r="A217" s="1" t="s">
+        <v>1490</v>
+      </c>
+      <c r="B217" s="1">
+        <v>106</v>
+      </c>
+      <c r="C217" s="1">
+        <v>7489</v>
+      </c>
+      <c r="D217" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E217" s="1">
+        <v>508</v>
+      </c>
+      <c r="F217" s="1">
+        <v>20</v>
+      </c>
+      <c r="G217" s="1">
+        <v>20</v>
+      </c>
+      <c r="H217" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8">
+      <c r="A218" s="1" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B218" s="1">
+        <v>106</v>
+      </c>
+      <c r="C218" s="1">
+        <v>7563</v>
+      </c>
+      <c r="D218" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E218" s="1">
+        <v>432</v>
+      </c>
+      <c r="F218" s="1">
+        <v>20</v>
+      </c>
+      <c r="G218" s="1">
+        <v>20</v>
+      </c>
+      <c r="H218" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8">
+      <c r="A219" s="1" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B219" s="1">
+        <v>106</v>
+      </c>
+      <c r="C219" s="1">
+        <v>7563</v>
+      </c>
+      <c r="D219" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E219" s="1">
+        <v>432</v>
+      </c>
+      <c r="F219" s="1">
+        <v>20</v>
+      </c>
+      <c r="G219" s="1">
+        <v>20</v>
+      </c>
+      <c r="H219" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8">
+      <c r="A220" s="1" t="s">
+        <v>1493</v>
+      </c>
+      <c r="B220" s="1">
+        <v>106</v>
+      </c>
+      <c r="C220" s="1">
+        <v>7538</v>
+      </c>
+      <c r="D220" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E220" s="1">
+        <v>356</v>
+      </c>
+      <c r="F220" s="1">
+        <v>20</v>
+      </c>
+      <c r="G220" s="1">
+        <v>20</v>
+      </c>
+      <c r="H220" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8">
+      <c r="A221" s="1" t="s">
+        <v>1494</v>
+      </c>
+      <c r="B221" s="1">
+        <v>106</v>
+      </c>
+      <c r="C221" s="1">
+        <v>7538</v>
+      </c>
+      <c r="D221" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E221" s="1">
+        <v>356</v>
+      </c>
+      <c r="F221" s="1">
+        <v>20</v>
+      </c>
+      <c r="G221" s="1">
+        <v>20</v>
+      </c>
+      <c r="H221" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8">
+      <c r="A222" s="1" t="s">
+        <v>1495</v>
+      </c>
+      <c r="B222" s="1">
+        <v>106</v>
+      </c>
+      <c r="C222" s="1">
+        <v>7698</v>
+      </c>
+      <c r="D222" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E222" s="1">
+        <v>298</v>
+      </c>
+      <c r="F222" s="1">
+        <v>20</v>
+      </c>
+      <c r="G222" s="1">
+        <v>20</v>
+      </c>
+      <c r="H222" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8">
+      <c r="A223" s="1" t="s">
+        <v>1496</v>
+      </c>
+      <c r="B223" s="1">
+        <v>106</v>
+      </c>
+      <c r="C223" s="1">
+        <v>7698</v>
+      </c>
+      <c r="D223" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E223" s="1">
+        <v>298</v>
+      </c>
+      <c r="F223" s="1">
+        <v>20</v>
+      </c>
+      <c r="G223" s="1">
+        <v>20</v>
+      </c>
+      <c r="H223" s="1">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cora banner + fix
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/neutralC.xlsx
+++ b/gu_in/Map.edf/neutralC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A54DC82D-7723-4D29-BA15-1FA79B8D3DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541A29A8-3718-4C85-A249-27048C2C3528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10965" yWindow="1020" windowWidth="10110" windowHeight="11205" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11730" yWindow="885" windowWidth="10110" windowHeight="11205" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3100" uniqueCount="1497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3108" uniqueCount="1505">
   <si>
     <t>char[32]</t>
   </si>
@@ -4529,6 +4529,30 @@
   </si>
   <si>
     <t>bd131C0</t>
+  </si>
+  <si>
+    <t>sd131C1</t>
+  </si>
+  <si>
+    <t>bd131C1</t>
+  </si>
+  <si>
+    <t>sd131C2</t>
+  </si>
+  <si>
+    <t>bd131C2</t>
+  </si>
+  <si>
+    <t>sd131C3</t>
+  </si>
+  <si>
+    <t>bd131C3</t>
+  </si>
+  <si>
+    <t>sd131C4</t>
+  </si>
+  <si>
+    <t>bd131C4</t>
   </si>
 </sst>
 </file>
@@ -46705,7 +46729,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H223"/>
+  <dimension ref="A1:H231"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="9.7109375" customWidth="1"/>
@@ -52413,13 +52437,13 @@
         <v>106</v>
       </c>
       <c r="C220" s="1">
-        <v>7538</v>
+        <v>7639</v>
       </c>
       <c r="D220" s="1">
         <v>-159</v>
       </c>
       <c r="E220" s="1">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F220" s="1">
         <v>20</v>
@@ -52439,13 +52463,13 @@
         <v>106</v>
       </c>
       <c r="C221" s="1">
-        <v>7538</v>
+        <v>7639</v>
       </c>
       <c r="D221" s="1">
         <v>-159</v>
       </c>
       <c r="E221" s="1">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F221" s="1">
         <v>20</v>
@@ -52506,6 +52530,214 @@
         <v>20</v>
       </c>
       <c r="H223" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8">
+      <c r="A224" s="1" t="s">
+        <v>1497</v>
+      </c>
+      <c r="B224" s="1">
+        <v>106</v>
+      </c>
+      <c r="C224" s="1">
+        <v>7313</v>
+      </c>
+      <c r="D224" s="1">
+        <v>-160</v>
+      </c>
+      <c r="E224" s="1">
+        <v>332</v>
+      </c>
+      <c r="F224" s="1">
+        <v>20</v>
+      </c>
+      <c r="G224" s="1">
+        <v>20</v>
+      </c>
+      <c r="H224" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8">
+      <c r="A225" s="1" t="s">
+        <v>1498</v>
+      </c>
+      <c r="B225" s="1">
+        <v>106</v>
+      </c>
+      <c r="C225" s="1">
+        <v>7313</v>
+      </c>
+      <c r="D225" s="1">
+        <v>-160</v>
+      </c>
+      <c r="E225" s="1">
+        <v>332</v>
+      </c>
+      <c r="F225" s="1">
+        <v>20</v>
+      </c>
+      <c r="G225" s="1">
+        <v>20</v>
+      </c>
+      <c r="H225" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8">
+      <c r="A226" s="1" t="s">
+        <v>1499</v>
+      </c>
+      <c r="B226" s="1">
+        <v>106</v>
+      </c>
+      <c r="C226" s="1">
+        <v>7388</v>
+      </c>
+      <c r="D226" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E226" s="1">
+        <v>258</v>
+      </c>
+      <c r="F226" s="1">
+        <v>20</v>
+      </c>
+      <c r="G226" s="1">
+        <v>20</v>
+      </c>
+      <c r="H226" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8">
+      <c r="A227" s="1" t="s">
+        <v>1500</v>
+      </c>
+      <c r="B227" s="1">
+        <v>106</v>
+      </c>
+      <c r="C227" s="1">
+        <v>7388</v>
+      </c>
+      <c r="D227" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E227" s="1">
+        <v>258</v>
+      </c>
+      <c r="F227" s="1">
+        <v>20</v>
+      </c>
+      <c r="G227" s="1">
+        <v>20</v>
+      </c>
+      <c r="H227" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8">
+      <c r="A228" s="1" t="s">
+        <v>1501</v>
+      </c>
+      <c r="B228" s="1">
+        <v>106</v>
+      </c>
+      <c r="C228" s="1">
+        <v>7463</v>
+      </c>
+      <c r="D228" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E228" s="1">
+        <v>183</v>
+      </c>
+      <c r="F228" s="1">
+        <v>20</v>
+      </c>
+      <c r="G228" s="1">
+        <v>20</v>
+      </c>
+      <c r="H228" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8">
+      <c r="A229" s="1" t="s">
+        <v>1502</v>
+      </c>
+      <c r="B229" s="1">
+        <v>106</v>
+      </c>
+      <c r="C229" s="1">
+        <v>7463</v>
+      </c>
+      <c r="D229" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E229" s="1">
+        <v>183</v>
+      </c>
+      <c r="F229" s="1">
+        <v>20</v>
+      </c>
+      <c r="G229" s="1">
+        <v>20</v>
+      </c>
+      <c r="H229" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8">
+      <c r="A230" s="1" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B230" s="1">
+        <v>106</v>
+      </c>
+      <c r="C230" s="1">
+        <v>7523</v>
+      </c>
+      <c r="D230" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E230" s="1">
+        <v>124</v>
+      </c>
+      <c r="F230" s="1">
+        <v>20</v>
+      </c>
+      <c r="G230" s="1">
+        <v>20</v>
+      </c>
+      <c r="H230" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8">
+      <c r="A231" s="1" t="s">
+        <v>1504</v>
+      </c>
+      <c r="B231" s="1">
+        <v>106</v>
+      </c>
+      <c r="C231" s="1">
+        <v>7523</v>
+      </c>
+      <c r="D231" s="1">
+        <v>-159</v>
+      </c>
+      <c r="E231" s="1">
+        <v>124</v>
+      </c>
+      <c r="F231" s="1">
+        <v>20</v>
+      </c>
+      <c r="G231" s="1">
+        <v>20</v>
+      </c>
+      <c r="H231" s="1">
         <v>20</v>
       </c>
     </row>

</xml_diff>